<commit_message>
Add cumulative hospitalization balance and clinical sources
</commit_message>
<xml_diff>
--- a/public/Plantilla_Balance_Hidrico_Enfermeria.xlsx
+++ b/public/Plantilla_Balance_Hidrico_Enfermeria.xlsx
@@ -2,10 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro" sheetId="1" r:id="Rb70aaf7b06eb4a3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="2" r:id="R71b6cf9ad6714d9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="3" r:id="R8594892dbc6f4298"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="4" r:id="R9eb39ce622974c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro" sheetId="1" r:id="Ra38f90222c6f4f87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="2" r:id="R516c1723d427435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="3" r:id="R84bf2af8ba454a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="4" r:id="Rf7ed54af1b824265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BH Acumulado" sheetId="5" r:id="R3db7703eb0a0433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bibliografia" sheetId="6" r:id="Rd8149ce0d5fe48a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +15,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={6B9DEC65-90CE-668D-0226-17BF861CB003}</x:author>
+    <x:author>tc={A4AD2E24-73D8-A971-D052-8BE95B41A18D}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="G10" authorId="0">
@@ -33,7 +35,7 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={27A82070-9E76-C6F3-16B3-0B151B5C1140}</x:author>
+    <x:author>tc={61FA2C08-A585-866B-BE5F-5F63A6A73256}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B10" authorId="0">
@@ -66,7 +68,7 @@
     <x:numFmt numFmtId="206" formatCode="#,##0"/>
     <x:numFmt numFmtId="207" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -134,6 +136,23 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FF8A4B18"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17313B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17313B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17313B"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -377,7 +396,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="124">
+  <x:cellXfs count="165">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -603,6 +622,101 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -849,6 +963,209 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Tendencia diaria y balance acumulado (mL)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Ingresos (mL)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'BH Acumulado'!$A$7:$A$36</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'BH Acumulado'!$B$7:$B$36</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0" mL"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Egresos (mL)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'BH Acumulado'!$A$7:$A$36</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'BH Acumulado'!$C$7:$C$36</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0" mL"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Balance diario (mL)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'BH Acumulado'!$A$7:$A$36</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'BH Acumulado'!$D$7:$D$36</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0" mL"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>BH acumulado (mL)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'BH Acumulado'!$A$7:$A$36</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'BH Acumulado'!$E$7:$E$36</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0" mL"</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:smooth val="0"/>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -875,7 +1192,42 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra2046ba3c2e34633"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7e330c25097450f"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3dd0a1691b6e4a10"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -886,7 +1238,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{7F6766A5-46FB-465F-84EF-0E3D00B5307A}"/>
+  <xltc:person displayName="User" id="{BF53F8F1-7323-4239-9D2D-F2EE39971DB7}"/>
 </xltc:personList>
 </file>
 
@@ -1083,7 +1435,7 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="G10" dT="2026-08-15T04:17:52.787" personId="{7F6766A5-46FB-465F-84EF-0E3D00B5307A}" id="{6B9DEC65-90CE-668D-0226-17BF861CB003}">
+  <xltc:threadedComment ref="G10" dT="2026-08-15T04:29:12.559" personId="{BF53F8F1-7323-4239-9D2D-F2EE39971DB7}" id="{A4AD2E24-73D8-A971-D052-8BE95B41A18D}">
     <xltc:text>Ingrese el volumen numérico en mililitros. No escriba la unidad dentro de la celda.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -1091,7 +1443,7 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B10" dT="2026-08-15T04:17:52.787" personId="{7F6766A5-46FB-465F-84EF-0E3D00B5307A}" id="{27A82070-9E76-C6F3-16B3-0B151B5C1140}">
+  <xltc:threadedComment ref="B10" dT="2026-08-15T04:29:12.56" personId="{BF53F8F1-7323-4239-9D2D-F2EE39971DB7}" id="{61FA2C08-A585-866B-BE5F-5F63A6A73256}">
     <xltc:text>Indicador informativo: diuresis total ÷ peso ÷ horas registradas. Interpretar según edad, contexto y protocolo institucional.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2333,7 +2685,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcccad19c075d4f03"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a565f2cd97e4e02"/>
 </x:worksheet>
 </file>
 
@@ -2584,7 +2936,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9bfa713c367431a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92e8c463f7914043"/>
 </x:worksheet>
 </file>
 
@@ -2899,7 +3251,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284fa25ad2c54dff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65eea91b959f488f"/>
 </x:worksheet>
 </file>
 
@@ -2919,7 +3271,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>GUÍA RÁPIDA · QUICK GUIDE · GUIA RÁPIDO</x:v>
+        <x:v>GUÍA RÁPIDA · QUICK GUIDE · 快速指南 · GUIA RÁPIDO</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -3015,7 +3367,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="119" t="str">
-        <x:v>PORTUGUÊS</x:v>
+        <x:v>简体中文</x:v>
       </x:c>
       <x:c r="B10" s="119" t="str"/>
       <x:c r="C10" s="119" t="str"/>
@@ -3027,7 +3379,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="118" t="str">
-        <x:v>1. Preencha os dados do paciente nas células amarelas.</x:v>
+        <x:v>1. 在黄色单元格中填写患者资料。</x:v>
       </x:c>
       <x:c r="B11" s="118" t="str"/>
       <x:c r="C11" s="118" t="str"/>
@@ -3039,7 +3391,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="118" t="str">
-        <x:v>2. Registre cada entrada ou saída em uma linha, sempre em mL.</x:v>
+        <x:v>2. 每行记录一次液体摄入或排出，统一使用 mL。</x:v>
       </x:c>
       <x:c r="B12" s="118" t="str"/>
       <x:c r="C12" s="118" t="str"/>
@@ -3049,48 +3401,94 @@
       <x:c r="G12" s="118" t="str"/>
       <x:c r="H12" s="118" t="str"/>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="119" t="str">
+        <x:v>PORTUGUÊS</x:v>
+      </x:c>
+      <x:c r="B13" s="119" t="str"/>
+      <x:c r="C13" s="119" t="str"/>
+      <x:c r="D13" s="119" t="str"/>
+      <x:c r="E13" s="119" t="str"/>
+      <x:c r="F13" s="119" t="str"/>
+      <x:c r="G13" s="119" t="str"/>
+      <x:c r="H13" s="119" t="str"/>
+    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="123" t="str">
-        <x:v>Seguridad / Safety / Segurança
-Verifique siempre los datos originales y aplique el protocolo de su institución. No use esta herramienta como única base para decisiones clínicas.</x:v>
-      </x:c>
-      <x:c r="B14" s="123"/>
-      <x:c r="C14" s="123"/>
-      <x:c r="D14" s="123"/>
-      <x:c r="E14" s="123"/>
-      <x:c r="F14" s="123"/>
-      <x:c r="G14" s="123"/>
-      <x:c r="H14" s="123"/>
+      <x:c r="A14" s="118" t="str">
+        <x:v>1. Preencha os dados do paciente nas células amarelas.</x:v>
+      </x:c>
+      <x:c r="B14" s="118" t="str"/>
+      <x:c r="C14" s="118" t="str"/>
+      <x:c r="D14" s="118" t="str"/>
+      <x:c r="E14" s="118" t="str"/>
+      <x:c r="F14" s="118" t="str"/>
+      <x:c r="G14" s="118" t="str"/>
+      <x:c r="H14" s="118" t="str"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="123"/>
-      <x:c r="B15" s="123"/>
-      <x:c r="C15" s="123"/>
-      <x:c r="D15" s="123"/>
-      <x:c r="E15" s="123"/>
-      <x:c r="F15" s="123"/>
-      <x:c r="G15" s="123"/>
-      <x:c r="H15" s="123"/>
+      <x:c r="A15" s="118" t="str">
+        <x:v>2. Registre cada entrada ou saída em uma linha, sempre em mL.</x:v>
+      </x:c>
+      <x:c r="B15" s="118" t="str"/>
+      <x:c r="C15" s="118" t="str"/>
+      <x:c r="D15" s="118" t="str"/>
+      <x:c r="E15" s="118" t="str"/>
+      <x:c r="F15" s="118" t="str"/>
+      <x:c r="G15" s="118" t="str"/>
+      <x:c r="H15" s="118" t="str"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="123"/>
-      <x:c r="B16" s="123"/>
-      <x:c r="C16" s="123"/>
-      <x:c r="D16" s="123"/>
-      <x:c r="E16" s="123"/>
-      <x:c r="F16" s="123"/>
-      <x:c r="G16" s="123"/>
-      <x:c r="H16" s="123"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="123"/>
-      <x:c r="B17" s="123"/>
-      <x:c r="C17" s="123"/>
-      <x:c r="D17" s="123"/>
-      <x:c r="E17" s="123"/>
-      <x:c r="F17" s="123"/>
-      <x:c r="G17" s="123"/>
-      <x:c r="H17" s="123"/>
+      <x:c r="A16" s="118"/>
+      <x:c r="B16" s="118"/>
+      <x:c r="C16" s="118"/>
+      <x:c r="D16" s="118"/>
+      <x:c r="E16" s="118"/>
+      <x:c r="F16" s="118"/>
+      <x:c r="G16" s="118"/>
+      <x:c r="H16" s="118"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="123" t="str">
+        <x:v>Seguridad / Safety / 安全 / Segurança
+Verifique siempre los datos originales y aplique el protocolo de su institución. Esta herramienta no sustituye la valoración ni el juicio clínico.</x:v>
+      </x:c>
+      <x:c r="B18" s="123"/>
+      <x:c r="C18" s="123"/>
+      <x:c r="D18" s="123"/>
+      <x:c r="E18" s="123"/>
+      <x:c r="F18" s="123"/>
+      <x:c r="G18" s="123"/>
+      <x:c r="H18" s="123"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="123"/>
+      <x:c r="B19" s="123"/>
+      <x:c r="C19" s="123"/>
+      <x:c r="D19" s="123"/>
+      <x:c r="E19" s="123"/>
+      <x:c r="F19" s="123"/>
+      <x:c r="G19" s="123"/>
+      <x:c r="H19" s="123"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="123"/>
+      <x:c r="B20" s="123"/>
+      <x:c r="C20" s="123"/>
+      <x:c r="D20" s="123"/>
+      <x:c r="E20" s="123"/>
+      <x:c r="F20" s="123"/>
+      <x:c r="G20" s="123"/>
+      <x:c r="H20" s="123"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="123"/>
+      <x:c r="B21" s="123"/>
+      <x:c r="C21" s="123"/>
+      <x:c r="D21" s="123"/>
+      <x:c r="E21" s="123"/>
+      <x:c r="F21" s="123"/>
+      <x:c r="G21" s="123"/>
+      <x:c r="H21" s="123"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3105,7 +3503,776 @@
     <x:mergeCell ref="A10:H10"/>
     <x:mergeCell ref="A11:H11"/>
     <x:mergeCell ref="A12:H12"/>
-    <x:mergeCell ref="A14:H17"/>
+    <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A14:H14"/>
+    <x:mergeCell ref="A15:H15"/>
+    <x:mergeCell ref="A16:H16"/>
+    <x:mergeCell ref="A18:H21"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>BALANCE HÍDRICO ACUMULADO · HOSPITALIZACIÓN</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="126" t="str">
+        <x:v>Registre o pegue un resumen por día. El balance diario es ingresos − egresos; el acumulado suma los balances desde el primer día de hospitalización.</x:v>
+      </x:c>
+      <x:c r="B3" s="126"/>
+      <x:c r="C3" s="126"/>
+      <x:c r="D3" s="126"/>
+      <x:c r="E3" s="126"/>
+      <x:c r="F3" s="126"/>
+      <x:c r="G3" s="126"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="126"/>
+      <x:c r="B4" s="126"/>
+      <x:c r="C4" s="126"/>
+      <x:c r="D4" s="126"/>
+      <x:c r="E4" s="126"/>
+      <x:c r="F4" s="126"/>
+      <x:c r="G4" s="126"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="17" t="str">
+        <x:v>Fecha</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Ingresos (mL)</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>Egresos (mL)</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>Balance diario (mL)</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
+        <x:v>BH acumulado (mL)</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
+        <x:v>Diuresis (mL/kg/h)</x:v>
+      </x:c>
+      <x:c r="G6" s="17" t="str">
+        <x:v>Observaciones</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="32"/>
+      <x:c r="B7" s="38"/>
+      <x:c r="C7" s="38"/>
+      <x:c r="D7" s="39" t="n">
+        <x:f>B7-C7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="39" t="n">
+        <x:f>D7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="127"/>
+      <x:c r="G7" s="23"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="33"/>
+      <x:c r="B8" s="40"/>
+      <x:c r="C8" s="40"/>
+      <x:c r="D8" s="41" t="n">
+        <x:f>B8-C8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="41" t="n">
+        <x:f>E7+D8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="128"/>
+      <x:c r="G8" s="27"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="33"/>
+      <x:c r="B9" s="40"/>
+      <x:c r="C9" s="40"/>
+      <x:c r="D9" s="41" t="n">
+        <x:f>B9-C9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="41" t="n">
+        <x:f>E8+D9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="128"/>
+      <x:c r="G9" s="27"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="33"/>
+      <x:c r="B10" s="40"/>
+      <x:c r="C10" s="40"/>
+      <x:c r="D10" s="41" t="n">
+        <x:f>B10-C10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="41" t="n">
+        <x:f>E9+D10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="128"/>
+      <x:c r="G10" s="27"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="33"/>
+      <x:c r="B11" s="40"/>
+      <x:c r="C11" s="40"/>
+      <x:c r="D11" s="41" t="n">
+        <x:f>B11-C11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="41" t="n">
+        <x:f>E10+D11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="128"/>
+      <x:c r="G11" s="27"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="33"/>
+      <x:c r="B12" s="40"/>
+      <x:c r="C12" s="40"/>
+      <x:c r="D12" s="41" t="n">
+        <x:f>B12-C12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="41" t="n">
+        <x:f>E11+D12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="128"/>
+      <x:c r="G12" s="27"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="33"/>
+      <x:c r="B13" s="40"/>
+      <x:c r="C13" s="40"/>
+      <x:c r="D13" s="41" t="n">
+        <x:f>B13-C13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="41" t="n">
+        <x:f>E12+D13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="128"/>
+      <x:c r="G13" s="27"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="33"/>
+      <x:c r="B14" s="40"/>
+      <x:c r="C14" s="40"/>
+      <x:c r="D14" s="41" t="n">
+        <x:f>B14-C14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="41" t="n">
+        <x:f>E13+D14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="128"/>
+      <x:c r="G14" s="27"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="33"/>
+      <x:c r="B15" s="40"/>
+      <x:c r="C15" s="40"/>
+      <x:c r="D15" s="41" t="n">
+        <x:f>B15-C15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="41" t="n">
+        <x:f>E14+D15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="128"/>
+      <x:c r="G15" s="27"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="33"/>
+      <x:c r="B16" s="40"/>
+      <x:c r="C16" s="40"/>
+      <x:c r="D16" s="41" t="n">
+        <x:f>B16-C16</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="41" t="n">
+        <x:f>E15+D16</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="128"/>
+      <x:c r="G16" s="27"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="33"/>
+      <x:c r="B17" s="40"/>
+      <x:c r="C17" s="40"/>
+      <x:c r="D17" s="41" t="n">
+        <x:f>B17-C17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="41" t="n">
+        <x:f>E16+D17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="128"/>
+      <x:c r="G17" s="27"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="33"/>
+      <x:c r="B18" s="40"/>
+      <x:c r="C18" s="40"/>
+      <x:c r="D18" s="41" t="n">
+        <x:f>B18-C18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="41" t="n">
+        <x:f>E17+D18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="128"/>
+      <x:c r="G18" s="27"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="33"/>
+      <x:c r="B19" s="40"/>
+      <x:c r="C19" s="40"/>
+      <x:c r="D19" s="41" t="n">
+        <x:f>B19-C19</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="41" t="n">
+        <x:f>E18+D19</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="128"/>
+      <x:c r="G19" s="27"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="33"/>
+      <x:c r="B20" s="40"/>
+      <x:c r="C20" s="40"/>
+      <x:c r="D20" s="41" t="n">
+        <x:f>B20-C20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="41" t="n">
+        <x:f>E19+D20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="128"/>
+      <x:c r="G20" s="27"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="33"/>
+      <x:c r="B21" s="40"/>
+      <x:c r="C21" s="40"/>
+      <x:c r="D21" s="41" t="n">
+        <x:f>B21-C21</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="41" t="n">
+        <x:f>E20+D21</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="128"/>
+      <x:c r="G21" s="27"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="33"/>
+      <x:c r="B22" s="40"/>
+      <x:c r="C22" s="40"/>
+      <x:c r="D22" s="41" t="n">
+        <x:f>B22-C22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="41" t="n">
+        <x:f>E21+D22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="128"/>
+      <x:c r="G22" s="27"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="33"/>
+      <x:c r="B23" s="40"/>
+      <x:c r="C23" s="40"/>
+      <x:c r="D23" s="41" t="n">
+        <x:f>B23-C23</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="41" t="n">
+        <x:f>E22+D23</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="128"/>
+      <x:c r="G23" s="27"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="33"/>
+      <x:c r="B24" s="40"/>
+      <x:c r="C24" s="40"/>
+      <x:c r="D24" s="41" t="n">
+        <x:f>B24-C24</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="41" t="n">
+        <x:f>E23+D24</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="128"/>
+      <x:c r="G24" s="27"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="33"/>
+      <x:c r="B25" s="40"/>
+      <x:c r="C25" s="40"/>
+      <x:c r="D25" s="41" t="n">
+        <x:f>B25-C25</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E25" s="41" t="n">
+        <x:f>E24+D25</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F25" s="128"/>
+      <x:c r="G25" s="27"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="33"/>
+      <x:c r="B26" s="40"/>
+      <x:c r="C26" s="40"/>
+      <x:c r="D26" s="41" t="n">
+        <x:f>B26-C26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="41" t="n">
+        <x:f>E25+D26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="128"/>
+      <x:c r="G26" s="27"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="33"/>
+      <x:c r="B27" s="40"/>
+      <x:c r="C27" s="40"/>
+      <x:c r="D27" s="41" t="n">
+        <x:f>B27-C27</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="41" t="n">
+        <x:f>E26+D27</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="128"/>
+      <x:c r="G27" s="27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="33"/>
+      <x:c r="B28" s="40"/>
+      <x:c r="C28" s="40"/>
+      <x:c r="D28" s="41" t="n">
+        <x:f>B28-C28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="41" t="n">
+        <x:f>E27+D28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F28" s="128"/>
+      <x:c r="G28" s="27"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="33"/>
+      <x:c r="B29" s="40"/>
+      <x:c r="C29" s="40"/>
+      <x:c r="D29" s="41" t="n">
+        <x:f>B29-C29</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="41" t="n">
+        <x:f>E28+D29</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="128"/>
+      <x:c r="G29" s="27"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="33"/>
+      <x:c r="B30" s="40"/>
+      <x:c r="C30" s="40"/>
+      <x:c r="D30" s="41" t="n">
+        <x:f>B30-C30</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="41" t="n">
+        <x:f>E29+D30</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" s="128"/>
+      <x:c r="G30" s="27"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="33"/>
+      <x:c r="B31" s="40"/>
+      <x:c r="C31" s="40"/>
+      <x:c r="D31" s="41" t="n">
+        <x:f>B31-C31</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="41" t="n">
+        <x:f>E30+D31</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="128"/>
+      <x:c r="G31" s="27"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="33"/>
+      <x:c r="B32" s="40"/>
+      <x:c r="C32" s="40"/>
+      <x:c r="D32" s="41" t="n">
+        <x:f>B32-C32</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="41" t="n">
+        <x:f>E31+D32</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="128"/>
+      <x:c r="G32" s="27"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="33"/>
+      <x:c r="B33" s="40"/>
+      <x:c r="C33" s="40"/>
+      <x:c r="D33" s="41" t="n">
+        <x:f>B33-C33</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="41" t="n">
+        <x:f>E32+D33</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F33" s="128"/>
+      <x:c r="G33" s="27"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="33"/>
+      <x:c r="B34" s="40"/>
+      <x:c r="C34" s="40"/>
+      <x:c r="D34" s="41" t="n">
+        <x:f>B34-C34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="41" t="n">
+        <x:f>E33+D34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" s="128"/>
+      <x:c r="G34" s="27"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="33"/>
+      <x:c r="B35" s="40"/>
+      <x:c r="C35" s="40"/>
+      <x:c r="D35" s="41" t="n">
+        <x:f>B35-C35</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="41" t="n">
+        <x:f>E34+D35</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="128"/>
+      <x:c r="G35" s="27"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="34"/>
+      <x:c r="B36" s="42"/>
+      <x:c r="C36" s="42"/>
+      <x:c r="D36" s="43" t="n">
+        <x:f>B36-C36</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="43" t="n">
+        <x:f>E35+D36</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F36" s="129"/>
+      <x:c r="G36" s="31"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A3:G4"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2c2c993b1f84d37"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="45" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>SUSTENTO DE CÁLCULOS Y BIBLIOGRAFÍA</x:v>
+      </x:c>
+      <x:c r="B1" s="3"/>
+      <x:c r="C1" s="3"/>
+      <x:c r="D1" s="3"/>
+      <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Resultado</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="str">
+        <x:v>Fórmula</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="str">
+        <x:v>Significado</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str">
+        <x:v>Sustento</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="str">
+        <x:v>Fuente oficial</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="153" t="str">
+        <x:v>Total de ingresos</x:v>
+      </x:c>
+      <x:c r="B4" s="154" t="str">
+        <x:v>Suma de todos los volúmenes clasificados como ingreso</x:v>
+      </x:c>
+      <x:c r="C4" s="154" t="str">
+        <x:v>Cantidad total administrada o ingerida en el período</x:v>
+      </x:c>
+      <x:c r="D4" s="154" t="str">
+        <x:v>mL</x:v>
+      </x:c>
+      <x:c r="E4" s="154" t="str">
+        <x:v>El registro debe incluir tipo y volumen de cada ingreso.</x:v>
+      </x:c>
+      <x:c r="F4" s="155" t="str">
+        <x:v>https://www.nice.org.uk/guidance/cg174/chapter/recommendations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="156" t="str">
+        <x:v>Total de egresos</x:v>
+      </x:c>
+      <x:c r="B5" s="157" t="str">
+        <x:v>Suma de todos los volúmenes clasificados como egreso</x:v>
+      </x:c>
+      <x:c r="C5" s="157" t="str">
+        <x:v>Cantidad total eliminada o medida en el período</x:v>
+      </x:c>
+      <x:c r="D5" s="157" t="str">
+        <x:v>mL</x:v>
+      </x:c>
+      <x:c r="E5" s="157" t="str">
+        <x:v>La monitorización incluye diuresis y otras pérdidas medibles.</x:v>
+      </x:c>
+      <x:c r="F5" s="158" t="str">
+        <x:v>https://www.nice.org.uk/guidance/ng29/chapter/recommendations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="156" t="str">
+        <x:v>Balance neto</x:v>
+      </x:c>
+      <x:c r="B6" s="157" t="str">
+        <x:v>Total ingresos − Total egresos</x:v>
+      </x:c>
+      <x:c r="C6" s="157" t="str">
+        <x:v>Positivo si ingresó más; negativo si egresó más</x:v>
+      </x:c>
+      <x:c r="D6" s="157" t="str">
+        <x:v>mL</x:v>
+      </x:c>
+      <x:c r="E6" s="157" t="str">
+        <x:v>Es una diferencia aritmética; requiere interpretación clínica y tendencia.</x:v>
+      </x:c>
+      <x:c r="F6" s="158" t="str">
+        <x:v>https://www.nice.org.uk/guidance/cg174/resources/intravenous-fluid-therapy-in-adults-in-hospital-pdf-35109752233669</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="156" t="str">
+        <x:v>Diuresis horaria por peso</x:v>
+      </x:c>
+      <x:c r="B7" s="157" t="str">
+        <x:v>Diuresis total ÷ peso (kg) ÷ horas observadas</x:v>
+      </x:c>
+      <x:c r="C7" s="157" t="str">
+        <x:v>Normaliza la producción urinaria por peso y tiempo</x:v>
+      </x:c>
+      <x:c r="D7" s="157" t="str">
+        <x:v>mL/kg/h</x:v>
+      </x:c>
+      <x:c r="E7" s="157" t="str">
+        <x:v>NICE usa &lt;0.5 mL/kg/h como criterio de oliguria en riesgo de lesión renal aguda; no es diagnóstico aislado.</x:v>
+      </x:c>
+      <x:c r="F7" s="158" t="str">
+        <x:v>https://www.nice.org.uk/guidance/ng148/chapter/Recommendations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="156" t="str">
+        <x:v>BH acumulado</x:v>
+      </x:c>
+      <x:c r="B8" s="157" t="str">
+        <x:v>Suma progresiva de balances diarios</x:v>
+      </x:c>
+      <x:c r="C8" s="157" t="str">
+        <x:v>Balance neto consolidado desde el primer día registrado</x:v>
+      </x:c>
+      <x:c r="D8" s="157" t="str">
+        <x:v>mL</x:v>
+      </x:c>
+      <x:c r="E8" s="157" t="str">
+        <x:v>Permite seguir la tendencia durante la hospitalización; correlacionar con peso, examen y laboratorio.</x:v>
+      </x:c>
+      <x:c r="F8" s="158" t="str">
+        <x:v>https://www.nice.org.uk/guidance/cg174/chapter/recommendations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="156"/>
+      <x:c r="B9" s="157"/>
+      <x:c r="C9" s="157"/>
+      <x:c r="D9" s="157"/>
+      <x:c r="E9" s="157"/>
+      <x:c r="F9" s="158"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="159" t="str">
+        <x:v>Bibliografía</x:v>
+      </x:c>
+      <x:c r="B10" s="160" t="str">
+        <x:v>Institución</x:v>
+      </x:c>
+      <x:c r="C10" s="160" t="str">
+        <x:v>Documento</x:v>
+      </x:c>
+      <x:c r="D10" s="160" t="str">
+        <x:v>Alcance</x:v>
+      </x:c>
+      <x:c r="E10" s="160" t="str">
+        <x:v>Consulta</x:v>
+      </x:c>
+      <x:c r="F10" s="161" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="156" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B11" s="157" t="str">
+        <x:v>NICE</x:v>
+      </x:c>
+      <x:c r="C11" s="157" t="str">
+        <x:v>CG174: Intravenous fluid therapy in adults in hospital</x:v>
+      </x:c>
+      <x:c r="D11" s="157" t="str">
+        <x:v>Adultos hospitalizados; evaluación, prescripción y seguimiento.</x:v>
+      </x:c>
+      <x:c r="E11" s="157" t="str">
+        <x:v>2026-08-14</x:v>
+      </x:c>
+      <x:c r="F11" s="158" t="str">
+        <x:v>https://www.nice.org.uk/guidance/cg174</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="156" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B12" s="157" t="str">
+        <x:v>NICE</x:v>
+      </x:c>
+      <x:c r="C12" s="157" t="str">
+        <x:v>NG29: Intravenous fluid therapy in children and young people</x:v>
+      </x:c>
+      <x:c r="D12" s="157" t="str">
+        <x:v>Registro horario de ingresos, egresos y totales acumulados.</x:v>
+      </x:c>
+      <x:c r="E12" s="157" t="str">
+        <x:v>2026-08-14</x:v>
+      </x:c>
+      <x:c r="F12" s="158" t="str">
+        <x:v>https://www.nice.org.uk/guidance/ng29/chapter/recommendations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="162" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B13" s="163" t="str">
+        <x:v>NICE</x:v>
+      </x:c>
+      <x:c r="C13" s="163" t="str">
+        <x:v>NG148: Acute kidney injury</x:v>
+      </x:c>
+      <x:c r="D13" s="163" t="str">
+        <x:v>Reconocimiento de oliguria y necesidad de respuesta clínica.</x:v>
+      </x:c>
+      <x:c r="E13" s="163" t="str">
+        <x:v>2026-08-14</x:v>
+      </x:c>
+      <x:c r="F13" s="164" t="str">
+        <x:v>https://www.nice.org.uk/guidance/ng148/chapter/Recommendations</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>